<commit_message>
Cambios varios /04/- 1-do 9:53 PM
</commit_message>
<xml_diff>
--- a/docs/shm_pruebas_funcionales.xlsx
+++ b/docs/shm_pruebas_funcionales.xlsx
@@ -8,22 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SAN_PABLO\02_HHMM\Desarrollo\ADG_SHM\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB7B1446-6FD1-49DC-97F8-30F50DCF3D45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17DC10DD-DD62-4B0D-9B28-424954A9873A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="469" xr2:uid="{A2F8EE2C-4AA7-42D6-8E2C-02159C540554}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="469" activeTab="2" xr2:uid="{A2F8EE2C-4AA7-42D6-8E2C-02159C540554}"/>
   </bookViews>
   <sheets>
     <sheet name="Proceso" sheetId="11" r:id="rId1"/>
-    <sheet name="0" sheetId="10" r:id="rId2"/>
-    <sheet name="1" sheetId="1" r:id="rId3"/>
-    <sheet name="2" sheetId="2" r:id="rId4"/>
-    <sheet name="3" sheetId="3" r:id="rId5"/>
-    <sheet name="4" sheetId="4" r:id="rId6"/>
-    <sheet name="5" sheetId="5" r:id="rId7"/>
-    <sheet name="6" sheetId="6" r:id="rId8"/>
-    <sheet name="7" sheetId="7" r:id="rId9"/>
-    <sheet name="8" sheetId="8" r:id="rId10"/>
-    <sheet name="9" sheetId="9" r:id="rId11"/>
+    <sheet name="Hoja1" sheetId="12" r:id="rId2"/>
+    <sheet name="0" sheetId="10" r:id="rId3"/>
+    <sheet name="1" sheetId="1" r:id="rId4"/>
+    <sheet name="2" sheetId="2" r:id="rId5"/>
+    <sheet name="3" sheetId="3" r:id="rId6"/>
+    <sheet name="4" sheetId="4" r:id="rId7"/>
+    <sheet name="5" sheetId="5" r:id="rId8"/>
+    <sheet name="6" sheetId="6" r:id="rId9"/>
+    <sheet name="7" sheetId="7" r:id="rId10"/>
+    <sheet name="8" sheetId="8" r:id="rId11"/>
+    <sheet name="9" sheetId="9" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -49,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="76">
   <si>
     <t>ID</t>
   </si>
@@ -274,6 +275,9 @@
   </si>
   <si>
     <t>Sistema Workflow de Honorarios Médicos para las Compañías Médicas</t>
+  </si>
+  <si>
+    <t>ordenar en forma alfabetica</t>
   </si>
 </sst>
 </file>
@@ -480,15 +484,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>117231</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>21980</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>669289</xdr:colOff>
-      <xdr:row>66</xdr:row>
-      <xdr:rowOff>97018</xdr:rowOff>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>24520</xdr:colOff>
+      <xdr:row>67</xdr:row>
+      <xdr:rowOff>118998</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -511,8 +515,57 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="0"/>
+          <a:off x="117231" y="212480"/>
           <a:ext cx="18195289" cy="12670018"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>84571</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>151643</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagen 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{629E8640-9618-52B5-BE2E-D3D2740F7A9B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="762000" y="762000"/>
+          <a:ext cx="9228571" cy="6057143"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -850,6 +903,120 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D10FA7E4-9298-4212-91A4-2F25705AB213}">
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7.5703125" customWidth="1"/>
+    <col min="2" max="2" width="61.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.85546875" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" customWidth="1"/>
+    <col min="6" max="6" width="24" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="11"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="5"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="10"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="11"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="10"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="5"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="10"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="11"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="10"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F0340D5-A23E-40B3-9B62-8F074AF061F6}">
   <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -964,7 +1131,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D42C2C95-45F4-4DD2-87F4-DBCD6DB33305}">
   <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1069,6 +1236,22 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F344445D-B0DA-4B75-AAFB-57C889C2F2EB}">
+  <dimension ref="C38"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="38" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C38" t="s">
+        <v>75</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A18E3AAE-20E2-41E5-B4AD-6D2A9BAA4860}">
   <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1240,7 +1423,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EB39019-C7D6-48C0-B993-96C13816BB10}">
   <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1390,7 +1573,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35DB2204-BAB5-4CEF-8D1A-0A7FC554D1DF}">
   <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1515,7 +1698,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D3CE5EE-79AB-467C-B303-CF45FE3ECFB1}">
   <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1638,7 +1821,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4400608D-558F-41E9-B06E-0492BD60E2B3}">
   <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1762,7 +1945,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2611D0FC-17AD-4FF7-AEF6-BD004B41653C}">
   <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1901,7 +2084,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD4A2839-9926-4DBB-BD72-3612D6856F31}">
   <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2022,118 +2205,4 @@
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D10FA7E4-9298-4212-91A4-2F25705AB213}">
-  <dimension ref="A1:F10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="7.5703125" customWidth="1"/>
-    <col min="2" max="2" width="61.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.85546875" customWidth="1"/>
-    <col min="4" max="4" width="16.7109375" customWidth="1"/>
-    <col min="6" max="6" width="24" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="16" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="11"/>
-      <c r="B6" s="6"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="5"/>
-      <c r="B7" s="6"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="10"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="11"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="10"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="5"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="10"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="11"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="10"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>